<commit_message>
Adiciona crédito presumido de resíduos sólidos (Art. 170, LC 214/2025)
Inclui campo de entrada para aquisições de resíduos sólidos de catadores
incentivados e calcula o crédito presumido de CBS (7% fixo) e IBS
(escalonado 1,3% a 13%, 2029-2033) na aba de transição da Reforma.
Corrige também referências de célula fixas em 'Dados de Entrada' que
foram substituídas por referências dinâmicas, para suportar a nova linha.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018ED9zBe28yKRAx5U4xtcTG
</commit_message>
<xml_diff>
--- a/Precificacao_Tributaria_Reforma_2027_2033.xlsx
+++ b/Precificacao_Tributaria_Reforma_2027_2033.xlsx
@@ -1160,7 +1160,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:H35"/>
+  <dimension ref="B2:H37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -1436,102 +1436,88 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="20" customHeight="1">
-      <c r="B24" s="6" t="inlineStr">
+    <row r="23" ht="46" customHeight="1">
+      <c r="B23" s="9" t="inlineStr">
+        <is>
+          <t>Crédito Presumido – Resíduos Sólidos, CBS (Art. 170, LC 214/2025)</t>
+        </is>
+      </c>
+      <c r="C23" s="17" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="D23" s="16" t="inlineStr">
+        <is>
+          <t>Percentual fixo previsto em lei (7%) sobre aquisições de resíduos sólidos de coletores incentivados (catador pessoa física, cooperativa ou associação), para destinação final ambientalmente adequada. Vigora junto com a CBS (a partir de 2027). Exclusões no §3º do art. 170 (ex.: agrotóxicos, medicamentos, pilhas/baterias).</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="40" customHeight="1">
+      <c r="B24" s="9" t="inlineStr">
+        <is>
+          <t>Crédito Presumido – Resíduos Sólidos, IBS pleno (Art. 170, LC 214/2025)</t>
+        </is>
+      </c>
+      <c r="C24" s="17" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="D24" s="16" t="inlineStr">
+        <is>
+          <t>Percentual pleno (13%, a partir de 2033) sobre a mesma base. Escalonado de 1,3% (2029) a 13% (2033) na mesma proporção do cronograma de transição do IBS (aba usa o peso 'Novo Estadual/Municipal' da linha 3 abaixo para graduar automaticamente).</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="20" customHeight="1">
+      <c r="B26" s="6" t="inlineStr">
         <is>
           <t>3. CRONOGRAMA DE TRANSIÇÃO (EC 132/2023 e LC 214/2025)</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="30" customHeight="1">
-      <c r="B25" s="14" t="inlineStr">
+    <row r="27" ht="30" customHeight="1">
+      <c r="B27" s="14" t="inlineStr">
         <is>
           <t>Ano</t>
         </is>
       </c>
-      <c r="C25" s="14" t="inlineStr">
+      <c r="C27" s="14" t="inlineStr">
         <is>
           <t>% Antigo
 (PIS/COFINS)</t>
         </is>
       </c>
-      <c r="D25" s="14" t="inlineStr">
+      <c r="D27" s="14" t="inlineStr">
         <is>
           <t>% Novo
 (CBS)</t>
         </is>
       </c>
-      <c r="E25" s="14" t="inlineStr">
+      <c r="E27" s="14" t="inlineStr">
         <is>
           <t>% Antigo
 (ICMS/ISS)</t>
         </is>
       </c>
-      <c r="F25" s="14" t="inlineStr">
+      <c r="F27" s="14" t="inlineStr">
         <is>
           <t>% Novo
 (IBS)</t>
         </is>
       </c>
-      <c r="G25" s="14" t="inlineStr">
+      <c r="G27" s="14" t="inlineStr">
         <is>
           <t>Observações</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="40" customHeight="1">
-      <c r="B26" s="20" t="n">
-        <v>2026</v>
-      </c>
-      <c r="C26" s="21" t="n">
-        <v>1</v>
-      </c>
-      <c r="D26" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="E26" s="21" t="n">
-        <v>1</v>
-      </c>
-      <c r="F26" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="G26" s="16" t="inlineStr">
-        <is>
-          <t>Ano-teste: CBS 0,9% e IBS 0,1% são compensáveis com PIS/COFINS/ICMS/ISS devidos (sem custo adicional líquido).</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="40" customHeight="1">
-      <c r="B27" s="20" t="n">
-        <v>2027</v>
-      </c>
-      <c r="C27" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="D27" s="21" t="n">
-        <v>1</v>
-      </c>
-      <c r="E27" s="21" t="n">
-        <v>1</v>
-      </c>
-      <c r="F27" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="G27" s="16" t="inlineStr">
-        <is>
-          <t>Extinção de PIS e COFINS; CBS em alíquota cheia. IPI reduzido a 0% (exceto Zona Franca de Manaus). IBS ainda em fase de teste (0,1%).</t>
         </is>
       </c>
     </row>
     <row r="28" ht="40" customHeight="1">
       <c r="B28" s="20" t="n">
-        <v>2028</v>
+        <v>2026</v>
       </c>
       <c r="C28" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="D28" s="21" t="n">
         <v>0</v>
-      </c>
-      <c r="D28" s="21" t="n">
-        <v>1</v>
       </c>
       <c r="E28" s="21" t="n">
         <v>1</v>
@@ -1541,13 +1527,13 @@
       </c>
       <c r="G28" s="16" t="inlineStr">
         <is>
-          <t>Mantém-se a sistemática de 2027 (CBS plena / ICMS-ISS integrais).</t>
+          <t>Ano-teste: CBS 0,9% e IBS 0,1% são compensáveis com PIS/COFINS/ICMS/ISS devidos (sem custo adicional líquido).</t>
         </is>
       </c>
     </row>
     <row r="29" ht="40" customHeight="1">
       <c r="B29" s="20" t="n">
-        <v>2029</v>
+        <v>2027</v>
       </c>
       <c r="C29" s="21" t="n">
         <v>0</v>
@@ -1556,20 +1542,20 @@
         <v>1</v>
       </c>
       <c r="E29" s="21" t="n">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="F29" s="21" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="G29" s="16" t="inlineStr">
         <is>
-          <t>Início da transição do IBS: redução de 10% em ICMS e ISS.</t>
+          <t>Extinção de PIS e COFINS; CBS em alíquota cheia. IPI reduzido a 0% (exceto Zona Franca de Manaus). IBS ainda em fase de teste (0,1%).</t>
         </is>
       </c>
     </row>
     <row r="30" ht="40" customHeight="1">
       <c r="B30" s="20" t="n">
-        <v>2030</v>
+        <v>2028</v>
       </c>
       <c r="C30" s="21" t="n">
         <v>0</v>
@@ -1578,20 +1564,20 @@
         <v>1</v>
       </c>
       <c r="E30" s="21" t="n">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="F30" s="21" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="G30" s="16" t="inlineStr">
         <is>
-          <t>Redução de 20% em ICMS e ISS.</t>
+          <t>Mantém-se a sistemática de 2027 (CBS plena / ICMS-ISS integrais).</t>
         </is>
       </c>
     </row>
     <row r="31" ht="40" customHeight="1">
       <c r="B31" s="20" t="n">
-        <v>2031</v>
+        <v>2029</v>
       </c>
       <c r="C31" s="21" t="n">
         <v>0</v>
@@ -1600,20 +1586,20 @@
         <v>1</v>
       </c>
       <c r="E31" s="21" t="n">
-        <v>0.7</v>
+        <v>0.9</v>
       </c>
       <c r="F31" s="21" t="n">
-        <v>0.3</v>
+        <v>0.1</v>
       </c>
       <c r="G31" s="16" t="inlineStr">
         <is>
-          <t>Redução de 30% em ICMS e ISS.</t>
+          <t>Início da transição do IBS: redução de 10% em ICMS e ISS.</t>
         </is>
       </c>
     </row>
     <row r="32" ht="40" customHeight="1">
       <c r="B32" s="20" t="n">
-        <v>2032</v>
+        <v>2030</v>
       </c>
       <c r="C32" s="21" t="n">
         <v>0</v>
@@ -1622,20 +1608,20 @@
         <v>1</v>
       </c>
       <c r="E32" s="21" t="n">
-        <v>0.6</v>
+        <v>0.8</v>
       </c>
       <c r="F32" s="21" t="n">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="G32" s="16" t="inlineStr">
         <is>
-          <t>Redução de 40% em ICMS e ISS.</t>
+          <t>Redução de 20% em ICMS e ISS.</t>
         </is>
       </c>
     </row>
     <row r="33" ht="40" customHeight="1">
       <c r="B33" s="20" t="n">
-        <v>2033</v>
+        <v>2031</v>
       </c>
       <c r="C33" s="21" t="n">
         <v>0</v>
@@ -1644,19 +1630,63 @@
         <v>1</v>
       </c>
       <c r="E33" s="21" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="F33" s="21" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="G33" s="16" t="inlineStr">
+        <is>
+          <t>Redução de 30% em ICMS e ISS.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="40" customHeight="1">
+      <c r="B34" s="20" t="n">
+        <v>2032</v>
+      </c>
+      <c r="C34" s="21" t="n">
         <v>0</v>
       </c>
-      <c r="F33" s="21" t="n">
+      <c r="D34" s="21" t="n">
         <v>1</v>
       </c>
-      <c r="G33" s="16" t="inlineStr">
+      <c r="E34" s="21" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="F34" s="21" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="G34" s="16" t="inlineStr">
+        <is>
+          <t>Redução de 40% em ICMS e ISS.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="40" customHeight="1">
+      <c r="B35" s="20" t="n">
+        <v>2033</v>
+      </c>
+      <c r="C35" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="D35" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="E35" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="F35" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="G35" s="16" t="inlineStr">
         <is>
           <t>Extinção total do ICMS e do ISS. IBS e CBS plenamente vigentes.</t>
         </is>
       </c>
     </row>
-    <row r="35" ht="30" customHeight="1">
-      <c r="B35" s="16" t="inlineStr">
+    <row r="37" ht="30" customHeight="1">
+      <c r="B37" s="16" t="inlineStr">
         <is>
           <t>Observação: os pesos acima refletem o desenho geral da transição previsto na EC 132/2023 e na LC 214/2025. Ajustes supervenientes por lei complementar/resolução devem ser refletidos diretamente nesta tabela.</t>
         </is>
@@ -1665,17 +1695,17 @@
   </sheetData>
   <mergeCells count="13">
     <mergeCell ref="G29:H29"/>
+    <mergeCell ref="G35:H35"/>
+    <mergeCell ref="G34:H34"/>
     <mergeCell ref="G30:H30"/>
-    <mergeCell ref="B35:H35"/>
     <mergeCell ref="G32:H32"/>
     <mergeCell ref="G33:H33"/>
     <mergeCell ref="B4:D4"/>
-    <mergeCell ref="G27:H27"/>
+    <mergeCell ref="B26:D26"/>
     <mergeCell ref="G28:H28"/>
     <mergeCell ref="G31:H31"/>
     <mergeCell ref="B15:D15"/>
-    <mergeCell ref="B24:D24"/>
-    <mergeCell ref="G26:H26"/>
+    <mergeCell ref="B37:H37"/>
     <mergeCell ref="B2:D2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1688,7 +1718,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:D23"/>
+  <dimension ref="B2:D25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -1810,116 +1840,148 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="20" customHeight="1">
-      <c r="B13" s="6" t="inlineStr">
+    <row r="12" ht="18" customHeight="1">
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>Adquire resíduos sólidos de catadores incentivados p/ destinação final adequada? (Sim/Não)</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="D12" s="19" t="inlineStr">
+        <is>
+          <t>Crédito presumido do Art. 170, LC 214/2025 (setor de reciclagem/sucata)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="20" customHeight="1">
+      <c r="B14" s="6" t="inlineStr">
         <is>
           <t>2. CUSTOS, DESPESAS E MARGEM</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="18" customHeight="1">
-      <c r="B14" s="9" t="inlineStr">
+    <row r="15" ht="18" customHeight="1">
+      <c r="B15" s="9" t="inlineStr">
         <is>
           <t>Custo de Aquisição/Produção Unitário (R$)</t>
         </is>
       </c>
-      <c r="C14" s="22" t="n">
+      <c r="C15" s="22" t="n">
         <v>100</v>
-      </c>
-    </row>
-    <row r="15" ht="26" customHeight="1">
-      <c r="B15" s="9" t="inlineStr">
-        <is>
-          <t>Insumos Sujeitos a Crédito Tributário (R$)</t>
-        </is>
-      </c>
-      <c r="C15" s="22" t="n">
-        <v>70</v>
-      </c>
-      <c r="D15" s="16" t="inlineStr">
-        <is>
-          <t>Parcela do custo acima referente a insumos com direito a crédito (compras de PJ, com nota fiscal).</t>
-        </is>
       </c>
     </row>
     <row r="16" ht="26" customHeight="1">
       <c r="B16" s="9" t="inlineStr">
         <is>
+          <t>Valor das Aquisições de Resíduos Sólidos de Catadores Incentivados (R$)</t>
+        </is>
+      </c>
+      <c r="C16" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="D16" s="16" t="inlineStr">
+        <is>
+          <t>Preencher somente se o campo acima for 'Sim'. Base de cálculo do crédito presumido do Art. 170, LC 214/2025.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="26" customHeight="1">
+      <c r="B17" s="9" t="inlineStr">
+        <is>
+          <t>Insumos Sujeitos a Crédito Tributário (R$)</t>
+        </is>
+      </c>
+      <c r="C17" s="22" t="n">
+        <v>70</v>
+      </c>
+      <c r="D17" s="16" t="inlineStr">
+        <is>
+          <t>Parcela do custo acima referente a insumos com direito a crédito (compras de PJ, com nota fiscal).</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="26" customHeight="1">
+      <c r="B18" s="9" t="inlineStr">
+        <is>
           <t>% de Aproveitamento do Crédito</t>
         </is>
       </c>
-      <c r="C16" s="21" t="n">
+      <c r="C18" s="21" t="n">
         <v>1</v>
       </c>
-      <c r="D16" s="16" t="inlineStr">
+      <c r="D18" s="16" t="inlineStr">
         <is>
           <t>100% para Lucro Real e Reforma (não cumulativo pleno); 0% para Simples/Presumido no regime atual.</t>
         </is>
-      </c>
-    </row>
-    <row r="17" ht="18" customHeight="1">
-      <c r="B17" s="9" t="inlineStr">
-        <is>
-          <t>Despesas Variáveis (%) — comissões, frete, cartão etc.</t>
-        </is>
-      </c>
-      <c r="C17" s="21" t="n">
-        <v>0.05</v>
-      </c>
-    </row>
-    <row r="18" ht="18" customHeight="1">
-      <c r="B18" s="9" t="inlineStr">
-        <is>
-          <t>Despesas Fixas Rateadas (%)</t>
-        </is>
-      </c>
-      <c r="C18" s="21" t="n">
-        <v>0.1</v>
       </c>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="B19" s="9" t="inlineStr">
         <is>
+          <t>Despesas Variáveis (%) — comissões, frete, cartão etc.</t>
+        </is>
+      </c>
+      <c r="C19" s="21" t="n">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="20" ht="18" customHeight="1">
+      <c r="B20" s="9" t="inlineStr">
+        <is>
+          <t>Despesas Fixas Rateadas (%)</t>
+        </is>
+      </c>
+      <c r="C20" s="21" t="n">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="21" ht="18" customHeight="1">
+      <c r="B21" s="9" t="inlineStr">
+        <is>
           <t>Margem de Lucro Desejada (%)</t>
         </is>
       </c>
-      <c r="C19" s="21" t="n">
+      <c r="C21" s="21" t="n">
         <v>0.2</v>
       </c>
     </row>
-    <row r="21" ht="20" customHeight="1">
-      <c r="B21" s="6" t="inlineStr">
+    <row r="23" ht="20" customHeight="1">
+      <c r="B23" s="6" t="inlineStr">
         <is>
           <t>3. RESUMO</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="B22" s="3" t="inlineStr">
+    <row r="24">
+      <c r="B24" s="3" t="inlineStr">
         <is>
           <t>Custo Total (base para formação de preço)</t>
         </is>
       </c>
-      <c r="C22" s="23">
-        <f>C14</f>
-        <v/>
-      </c>
-    </row>
-    <row r="23">
-      <c r="B23" s="3" t="inlineStr">
+      <c r="C24" s="23">
+        <f>C15</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" s="3" t="inlineStr">
         <is>
           <t>Soma Despesas Variáveis + Despesas Fixas + Margem</t>
         </is>
       </c>
-      <c r="C23" s="24">
-        <f>C17+C18+C19</f>
+      <c r="C25" s="24">
+        <f>C19+C20+C21</f>
         <v/>
       </c>
     </row>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="B21:D21"/>
-    <mergeCell ref="B13:D13"/>
+    <mergeCell ref="B23:D23"/>
+    <mergeCell ref="B14:D14"/>
     <mergeCell ref="B2:D2"/>
     <mergeCell ref="B4:D4"/>
   </mergeCells>
@@ -1930,7 +1992,7 @@
     <dataValidation sqref="C7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Simples Nacional,Lucro Presumido,Lucro Real"</formula1>
     </dataValidation>
-    <dataValidation sqref="C10 C11" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="C10 C11 C12" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Sim,Não"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2152,7 +2214,7 @@
         </is>
       </c>
       <c r="C24" s="28">
-        <f>'Dados de Entrada'!C15*'Dados de Entrada'!C16*C23</f>
+        <f>'Dados de Entrada'!C17*'Dados de Entrada'!C18*C23</f>
         <v/>
       </c>
       <c r="D24" s="16">
@@ -2230,7 +2292,7 @@
         </is>
       </c>
       <c r="C33" s="28">
-        <f>'Dados de Entrada'!C14-C28</f>
+        <f>'Dados de Entrada'!C15-C28</f>
         <v/>
       </c>
     </row>
@@ -2241,7 +2303,7 @@
         </is>
       </c>
       <c r="C34" s="29">
-        <f>1-('Dados de Entrada'!C17+'Dados de Entrada'!C18+'Dados de Entrada'!C19+C27)</f>
+        <f>1-('Dados de Entrada'!C19+'Dados de Entrada'!C20+'Dados de Entrada'!C21+C27)</f>
         <v/>
       </c>
     </row>
@@ -2274,7 +2336,7 @@
         </is>
       </c>
       <c r="C37" s="28">
-        <f>C35*'Dados de Entrada'!C19</f>
+        <f>C35*'Dados de Entrada'!C21</f>
         <v/>
       </c>
     </row>
@@ -2297,7 +2359,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:J26"/>
+  <dimension ref="B2:J31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -2339,35 +2401,35 @@
         </is>
       </c>
       <c r="C6" s="32">
-        <f>Parâmetros!B26</f>
+        <f>Parâmetros!B28</f>
         <v/>
       </c>
       <c r="D6" s="32">
-        <f>Parâmetros!B27</f>
+        <f>Parâmetros!B29</f>
         <v/>
       </c>
       <c r="E6" s="32">
-        <f>Parâmetros!B28</f>
+        <f>Parâmetros!B30</f>
         <v/>
       </c>
       <c r="F6" s="32">
-        <f>Parâmetros!B29</f>
+        <f>Parâmetros!B31</f>
         <v/>
       </c>
       <c r="G6" s="32">
-        <f>Parâmetros!B30</f>
+        <f>Parâmetros!B32</f>
         <v/>
       </c>
       <c r="H6" s="32">
-        <f>Parâmetros!B31</f>
+        <f>Parâmetros!B33</f>
         <v/>
       </c>
       <c r="I6" s="32">
-        <f>Parâmetros!B32</f>
+        <f>Parâmetros!B34</f>
         <v/>
       </c>
       <c r="J6" s="32">
-        <f>Parâmetros!B33</f>
+        <f>Parâmetros!B35</f>
         <v/>
       </c>
     </row>
@@ -2385,35 +2447,35 @@
         </is>
       </c>
       <c r="C8" s="34">
-        <f>Parâmetros!C26</f>
+        <f>Parâmetros!C28</f>
         <v/>
       </c>
       <c r="D8" s="34">
-        <f>Parâmetros!C27</f>
+        <f>Parâmetros!C29</f>
         <v/>
       </c>
       <c r="E8" s="34">
-        <f>Parâmetros!C28</f>
+        <f>Parâmetros!C30</f>
         <v/>
       </c>
       <c r="F8" s="34">
-        <f>Parâmetros!C29</f>
+        <f>Parâmetros!C31</f>
         <v/>
       </c>
       <c r="G8" s="34">
-        <f>Parâmetros!C30</f>
+        <f>Parâmetros!C32</f>
         <v/>
       </c>
       <c r="H8" s="34">
-        <f>Parâmetros!C31</f>
+        <f>Parâmetros!C33</f>
         <v/>
       </c>
       <c r="I8" s="34">
-        <f>Parâmetros!C32</f>
+        <f>Parâmetros!C34</f>
         <v/>
       </c>
       <c r="J8" s="34">
-        <f>Parâmetros!C33</f>
+        <f>Parâmetros!C35</f>
         <v/>
       </c>
     </row>
@@ -2424,35 +2486,35 @@
         </is>
       </c>
       <c r="C9" s="34">
-        <f>Parâmetros!D26</f>
+        <f>Parâmetros!D28</f>
         <v/>
       </c>
       <c r="D9" s="34">
-        <f>Parâmetros!D27</f>
+        <f>Parâmetros!D29</f>
         <v/>
       </c>
       <c r="E9" s="34">
-        <f>Parâmetros!D28</f>
+        <f>Parâmetros!D30</f>
         <v/>
       </c>
       <c r="F9" s="34">
-        <f>Parâmetros!D29</f>
+        <f>Parâmetros!D31</f>
         <v/>
       </c>
       <c r="G9" s="34">
-        <f>Parâmetros!D30</f>
+        <f>Parâmetros!D32</f>
         <v/>
       </c>
       <c r="H9" s="34">
-        <f>Parâmetros!D31</f>
+        <f>Parâmetros!D33</f>
         <v/>
       </c>
       <c r="I9" s="34">
-        <f>Parâmetros!D32</f>
+        <f>Parâmetros!D34</f>
         <v/>
       </c>
       <c r="J9" s="34">
-        <f>Parâmetros!D33</f>
+        <f>Parâmetros!D35</f>
         <v/>
       </c>
     </row>
@@ -2463,35 +2525,35 @@
         </is>
       </c>
       <c r="C10" s="34">
-        <f>Parâmetros!E26</f>
+        <f>Parâmetros!E28</f>
         <v/>
       </c>
       <c r="D10" s="34">
-        <f>Parâmetros!E27</f>
+        <f>Parâmetros!E29</f>
         <v/>
       </c>
       <c r="E10" s="34">
-        <f>Parâmetros!E28</f>
+        <f>Parâmetros!E30</f>
         <v/>
       </c>
       <c r="F10" s="34">
-        <f>Parâmetros!E29</f>
+        <f>Parâmetros!E31</f>
         <v/>
       </c>
       <c r="G10" s="34">
-        <f>Parâmetros!E30</f>
+        <f>Parâmetros!E32</f>
         <v/>
       </c>
       <c r="H10" s="34">
-        <f>Parâmetros!E31</f>
+        <f>Parâmetros!E33</f>
         <v/>
       </c>
       <c r="I10" s="34">
-        <f>Parâmetros!E32</f>
+        <f>Parâmetros!E34</f>
         <v/>
       </c>
       <c r="J10" s="34">
-        <f>Parâmetros!E33</f>
+        <f>Parâmetros!E35</f>
         <v/>
       </c>
     </row>
@@ -2502,35 +2564,35 @@
         </is>
       </c>
       <c r="C11" s="34">
-        <f>Parâmetros!F26</f>
+        <f>Parâmetros!F28</f>
         <v/>
       </c>
       <c r="D11" s="34">
-        <f>Parâmetros!F27</f>
+        <f>Parâmetros!F29</f>
         <v/>
       </c>
       <c r="E11" s="34">
-        <f>Parâmetros!F28</f>
+        <f>Parâmetros!F30</f>
         <v/>
       </c>
       <c r="F11" s="34">
-        <f>Parâmetros!F29</f>
+        <f>Parâmetros!F31</f>
         <v/>
       </c>
       <c r="G11" s="34">
-        <f>Parâmetros!F30</f>
+        <f>Parâmetros!F32</f>
         <v/>
       </c>
       <c r="H11" s="34">
-        <f>Parâmetros!F31</f>
+        <f>Parâmetros!F33</f>
         <v/>
       </c>
       <c r="I11" s="34">
-        <f>Parâmetros!F32</f>
+        <f>Parâmetros!F34</f>
         <v/>
       </c>
       <c r="J11" s="34">
-        <f>Parâmetros!F33</f>
+        <f>Parâmetros!F35</f>
         <v/>
       </c>
     </row>
@@ -2707,247 +2769,372 @@
     <row r="20" ht="20" customHeight="1">
       <c r="B20" s="6" t="inlineStr">
         <is>
-          <t>CRÉDITOS E FORMAÇÃO DE PREÇO</t>
+          <t>CRÉDITO PRESUMIDO — RESÍDUOS SÓLIDOS (ART. 170, LC 214/2025)</t>
         </is>
       </c>
     </row>
     <row r="21" ht="26" customHeight="1">
       <c r="B21" s="35" t="inlineStr">
         <is>
-          <t>Créditos Recuperáveis sobre Insumos (R$)</t>
+          <t>Crédito Presumido CBS (7% fixo, a partir de 2027)</t>
         </is>
       </c>
       <c r="C21" s="37">
-        <f>IF('Dados de Entrada'!$C$7="Simples Nacional",0,'Dados de Entrada'!$C$15*'Dados de Entrada'!$C$16*C17)</f>
+        <f>IF('Dados de Entrada'!$C$12="Sim",'Dados de Entrada'!$C$16*C9*Parâmetros!$C$23,0)</f>
         <v/>
       </c>
       <c r="D21" s="37">
-        <f>IF('Dados de Entrada'!$C$7="Simples Nacional",0,'Dados de Entrada'!$C$15*'Dados de Entrada'!$C$16*D17)</f>
+        <f>IF('Dados de Entrada'!$C$12="Sim",'Dados de Entrada'!$C$16*D9*Parâmetros!$C$23,0)</f>
         <v/>
       </c>
       <c r="E21" s="37">
-        <f>IF('Dados de Entrada'!$C$7="Simples Nacional",0,'Dados de Entrada'!$C$15*'Dados de Entrada'!$C$16*E17)</f>
+        <f>IF('Dados de Entrada'!$C$12="Sim",'Dados de Entrada'!$C$16*E9*Parâmetros!$C$23,0)</f>
         <v/>
       </c>
       <c r="F21" s="37">
-        <f>IF('Dados de Entrada'!$C$7="Simples Nacional",0,'Dados de Entrada'!$C$15*'Dados de Entrada'!$C$16*F17)</f>
+        <f>IF('Dados de Entrada'!$C$12="Sim",'Dados de Entrada'!$C$16*F9*Parâmetros!$C$23,0)</f>
         <v/>
       </c>
       <c r="G21" s="37">
-        <f>IF('Dados de Entrada'!$C$7="Simples Nacional",0,'Dados de Entrada'!$C$15*'Dados de Entrada'!$C$16*G17)</f>
+        <f>IF('Dados de Entrada'!$C$12="Sim",'Dados de Entrada'!$C$16*G9*Parâmetros!$C$23,0)</f>
         <v/>
       </c>
       <c r="H21" s="37">
-        <f>IF('Dados de Entrada'!$C$7="Simples Nacional",0,'Dados de Entrada'!$C$15*'Dados de Entrada'!$C$16*H17)</f>
+        <f>IF('Dados de Entrada'!$C$12="Sim",'Dados de Entrada'!$C$16*H9*Parâmetros!$C$23,0)</f>
         <v/>
       </c>
       <c r="I21" s="37">
-        <f>IF('Dados de Entrada'!$C$7="Simples Nacional",0,'Dados de Entrada'!$C$15*'Dados de Entrada'!$C$16*I17)</f>
+        <f>IF('Dados de Entrada'!$C$12="Sim",'Dados de Entrada'!$C$16*I9*Parâmetros!$C$23,0)</f>
         <v/>
       </c>
       <c r="J21" s="37">
-        <f>IF('Dados de Entrada'!$C$7="Simples Nacional",0,'Dados de Entrada'!$C$15*'Dados de Entrada'!$C$16*J17)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="22">
-      <c r="B22" s="33" t="inlineStr">
+        <f>IF('Dados de Entrada'!$C$12="Sim",'Dados de Entrada'!$C$16*J9*Parâmetros!$C$23,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22" ht="26" customHeight="1">
+      <c r="B22" s="35" t="inlineStr">
+        <is>
+          <t>Crédito Presumido IBS (escalonado 1,3%→13%, 2029-2033)</t>
+        </is>
+      </c>
+      <c r="C22" s="37">
+        <f>IF('Dados de Entrada'!$C$12="Sim",'Dados de Entrada'!$C$16*C11*Parâmetros!$C$24,0)</f>
+        <v/>
+      </c>
+      <c r="D22" s="37">
+        <f>IF('Dados de Entrada'!$C$12="Sim",'Dados de Entrada'!$C$16*D11*Parâmetros!$C$24,0)</f>
+        <v/>
+      </c>
+      <c r="E22" s="37">
+        <f>IF('Dados de Entrada'!$C$12="Sim",'Dados de Entrada'!$C$16*E11*Parâmetros!$C$24,0)</f>
+        <v/>
+      </c>
+      <c r="F22" s="37">
+        <f>IF('Dados de Entrada'!$C$12="Sim",'Dados de Entrada'!$C$16*F11*Parâmetros!$C$24,0)</f>
+        <v/>
+      </c>
+      <c r="G22" s="37">
+        <f>IF('Dados de Entrada'!$C$12="Sim",'Dados de Entrada'!$C$16*G11*Parâmetros!$C$24,0)</f>
+        <v/>
+      </c>
+      <c r="H22" s="37">
+        <f>IF('Dados de Entrada'!$C$12="Sim",'Dados de Entrada'!$C$16*H11*Parâmetros!$C$24,0)</f>
+        <v/>
+      </c>
+      <c r="I22" s="37">
+        <f>IF('Dados de Entrada'!$C$12="Sim",'Dados de Entrada'!$C$16*I11*Parâmetros!$C$24,0)</f>
+        <v/>
+      </c>
+      <c r="J22" s="37">
+        <f>IF('Dados de Entrada'!$C$12="Sim",'Dados de Entrada'!$C$16*J11*Parâmetros!$C$24,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>Total Crédito Presumido Art. 170 (R$)</t>
+        </is>
+      </c>
+      <c r="C23" s="38">
+        <f>C21+C22</f>
+        <v/>
+      </c>
+      <c r="D23" s="38">
+        <f>D21+D22</f>
+        <v/>
+      </c>
+      <c r="E23" s="38">
+        <f>E21+E22</f>
+        <v/>
+      </c>
+      <c r="F23" s="38">
+        <f>F21+F22</f>
+        <v/>
+      </c>
+      <c r="G23" s="38">
+        <f>G21+G22</f>
+        <v/>
+      </c>
+      <c r="H23" s="38">
+        <f>H21+H22</f>
+        <v/>
+      </c>
+      <c r="I23" s="38">
+        <f>I21+I22</f>
+        <v/>
+      </c>
+      <c r="J23" s="38">
+        <f>J21+J22</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25" ht="20" customHeight="1">
+      <c r="B25" s="6" t="inlineStr">
+        <is>
+          <t>CRÉDITOS E FORMAÇÃO DE PREÇO</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="26" customHeight="1">
+      <c r="B26" s="35" t="inlineStr">
+        <is>
+          <t>Créditos Recuperáveis Totais (Insumos + Art. 170) (R$)</t>
+        </is>
+      </c>
+      <c r="C26" s="37">
+        <f>IF('Dados de Entrada'!$C$7="Simples Nacional",0,'Dados de Entrada'!$C$17*'Dados de Entrada'!$C$18*C17)+C23</f>
+        <v/>
+      </c>
+      <c r="D26" s="37">
+        <f>IF('Dados de Entrada'!$C$7="Simples Nacional",0,'Dados de Entrada'!$C$17*'Dados de Entrada'!$C$18*D17)+D23</f>
+        <v/>
+      </c>
+      <c r="E26" s="37">
+        <f>IF('Dados de Entrada'!$C$7="Simples Nacional",0,'Dados de Entrada'!$C$17*'Dados de Entrada'!$C$18*E17)+E23</f>
+        <v/>
+      </c>
+      <c r="F26" s="37">
+        <f>IF('Dados de Entrada'!$C$7="Simples Nacional",0,'Dados de Entrada'!$C$17*'Dados de Entrada'!$C$18*F17)+F23</f>
+        <v/>
+      </c>
+      <c r="G26" s="37">
+        <f>IF('Dados de Entrada'!$C$7="Simples Nacional",0,'Dados de Entrada'!$C$17*'Dados de Entrada'!$C$18*G17)+G23</f>
+        <v/>
+      </c>
+      <c r="H26" s="37">
+        <f>IF('Dados de Entrada'!$C$7="Simples Nacional",0,'Dados de Entrada'!$C$17*'Dados de Entrada'!$C$18*H17)+H23</f>
+        <v/>
+      </c>
+      <c r="I26" s="37">
+        <f>IF('Dados de Entrada'!$C$7="Simples Nacional",0,'Dados de Entrada'!$C$17*'Dados de Entrada'!$C$18*I17)+I23</f>
+        <v/>
+      </c>
+      <c r="J26" s="37">
+        <f>IF('Dados de Entrada'!$C$7="Simples Nacional",0,'Dados de Entrada'!$C$17*'Dados de Entrada'!$C$18*J17)+J23</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" s="33" t="inlineStr">
         <is>
           <t>Custo Líquido de Créditos (R$)</t>
         </is>
       </c>
-      <c r="C22" s="37">
-        <f>'Dados de Entrada'!$C$14-C21</f>
-        <v/>
-      </c>
-      <c r="D22" s="37">
-        <f>'Dados de Entrada'!$C$14-D21</f>
-        <v/>
-      </c>
-      <c r="E22" s="37">
-        <f>'Dados de Entrada'!$C$14-E21</f>
-        <v/>
-      </c>
-      <c r="F22" s="37">
-        <f>'Dados de Entrada'!$C$14-F21</f>
-        <v/>
-      </c>
-      <c r="G22" s="37">
-        <f>'Dados de Entrada'!$C$14-G21</f>
-        <v/>
-      </c>
-      <c r="H22" s="37">
-        <f>'Dados de Entrada'!$C$14-H21</f>
-        <v/>
-      </c>
-      <c r="I22" s="37">
-        <f>'Dados de Entrada'!$C$14-I21</f>
-        <v/>
-      </c>
-      <c r="J22" s="37">
-        <f>'Dados de Entrada'!$C$14-J21</f>
-        <v/>
-      </c>
-    </row>
-    <row r="23" ht="26" customHeight="1">
-      <c r="B23" s="35" t="inlineStr">
+      <c r="C27" s="37">
+        <f>'Dados de Entrada'!$C$15-C26</f>
+        <v/>
+      </c>
+      <c r="D27" s="37">
+        <f>'Dados de Entrada'!$C$15-D26</f>
+        <v/>
+      </c>
+      <c r="E27" s="37">
+        <f>'Dados de Entrada'!$C$15-E26</f>
+        <v/>
+      </c>
+      <c r="F27" s="37">
+        <f>'Dados de Entrada'!$C$15-F26</f>
+        <v/>
+      </c>
+      <c r="G27" s="37">
+        <f>'Dados de Entrada'!$C$15-G26</f>
+        <v/>
+      </c>
+      <c r="H27" s="37">
+        <f>'Dados de Entrada'!$C$15-H26</f>
+        <v/>
+      </c>
+      <c r="I27" s="37">
+        <f>'Dados de Entrada'!$C$15-I26</f>
+        <v/>
+      </c>
+      <c r="J27" s="37">
+        <f>'Dados de Entrada'!$C$15-J26</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28" ht="26" customHeight="1">
+      <c r="B28" s="35" t="inlineStr">
         <is>
           <t>Divisor = 1 − (Desp.Var. + Desp.Fixas + Margem + Carga Total)</t>
         </is>
       </c>
-      <c r="C23" s="29">
-        <f>1-('Dados de Entrada'!$C$17+'Dados de Entrada'!$C$18+'Dados de Entrada'!$C$19+C17)</f>
-        <v/>
-      </c>
-      <c r="D23" s="29">
-        <f>1-('Dados de Entrada'!$C$17+'Dados de Entrada'!$C$18+'Dados de Entrada'!$C$19+D17)</f>
-        <v/>
-      </c>
-      <c r="E23" s="29">
-        <f>1-('Dados de Entrada'!$C$17+'Dados de Entrada'!$C$18+'Dados de Entrada'!$C$19+E17)</f>
-        <v/>
-      </c>
-      <c r="F23" s="29">
-        <f>1-('Dados de Entrada'!$C$17+'Dados de Entrada'!$C$18+'Dados de Entrada'!$C$19+F17)</f>
-        <v/>
-      </c>
-      <c r="G23" s="29">
-        <f>1-('Dados de Entrada'!$C$17+'Dados de Entrada'!$C$18+'Dados de Entrada'!$C$19+G17)</f>
-        <v/>
-      </c>
-      <c r="H23" s="29">
-        <f>1-('Dados de Entrada'!$C$17+'Dados de Entrada'!$C$18+'Dados de Entrada'!$C$19+H17)</f>
-        <v/>
-      </c>
-      <c r="I23" s="29">
-        <f>1-('Dados de Entrada'!$C$17+'Dados de Entrada'!$C$18+'Dados de Entrada'!$C$19+I17)</f>
-        <v/>
-      </c>
-      <c r="J23" s="29">
-        <f>1-('Dados de Entrada'!$C$17+'Dados de Entrada'!$C$18+'Dados de Entrada'!$C$19+J17)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="24">
-      <c r="B24" s="3" t="inlineStr">
+      <c r="C28" s="29">
+        <f>1-('Dados de Entrada'!$C$19+'Dados de Entrada'!$C$20+'Dados de Entrada'!$C$21+C17)</f>
+        <v/>
+      </c>
+      <c r="D28" s="29">
+        <f>1-('Dados de Entrada'!$C$19+'Dados de Entrada'!$C$20+'Dados de Entrada'!$C$21+D17)</f>
+        <v/>
+      </c>
+      <c r="E28" s="29">
+        <f>1-('Dados de Entrada'!$C$19+'Dados de Entrada'!$C$20+'Dados de Entrada'!$C$21+E17)</f>
+        <v/>
+      </c>
+      <c r="F28" s="29">
+        <f>1-('Dados de Entrada'!$C$19+'Dados de Entrada'!$C$20+'Dados de Entrada'!$C$21+F17)</f>
+        <v/>
+      </c>
+      <c r="G28" s="29">
+        <f>1-('Dados de Entrada'!$C$19+'Dados de Entrada'!$C$20+'Dados de Entrada'!$C$21+G17)</f>
+        <v/>
+      </c>
+      <c r="H28" s="29">
+        <f>1-('Dados de Entrada'!$C$19+'Dados de Entrada'!$C$20+'Dados de Entrada'!$C$21+H17)</f>
+        <v/>
+      </c>
+      <c r="I28" s="29">
+        <f>1-('Dados de Entrada'!$C$19+'Dados de Entrada'!$C$20+'Dados de Entrada'!$C$21+I17)</f>
+        <v/>
+      </c>
+      <c r="J28" s="29">
+        <f>1-('Dados de Entrada'!$C$19+'Dados de Entrada'!$C$20+'Dados de Entrada'!$C$21+J17)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" s="3" t="inlineStr">
         <is>
           <t>PREÇO DE VENDA NECESSÁRIO (R$)</t>
         </is>
       </c>
-      <c r="C24" s="38">
-        <f>C22/C23</f>
-        <v/>
-      </c>
-      <c r="D24" s="38">
-        <f>D22/D23</f>
-        <v/>
-      </c>
-      <c r="E24" s="38">
-        <f>E22/E23</f>
-        <v/>
-      </c>
-      <c r="F24" s="38">
-        <f>F22/F23</f>
-        <v/>
-      </c>
-      <c r="G24" s="38">
-        <f>G22/G23</f>
-        <v/>
-      </c>
-      <c r="H24" s="38">
-        <f>H22/H23</f>
-        <v/>
-      </c>
-      <c r="I24" s="38">
-        <f>I22/I23</f>
-        <v/>
-      </c>
-      <c r="J24" s="38">
-        <f>J22/J23</f>
-        <v/>
-      </c>
-    </row>
-    <row r="25">
-      <c r="B25" s="33" t="inlineStr">
+      <c r="C29" s="38">
+        <f>C27/C28</f>
+        <v/>
+      </c>
+      <c r="D29" s="38">
+        <f>D27/D28</f>
+        <v/>
+      </c>
+      <c r="E29" s="38">
+        <f>E27/E28</f>
+        <v/>
+      </c>
+      <c r="F29" s="38">
+        <f>F27/F28</f>
+        <v/>
+      </c>
+      <c r="G29" s="38">
+        <f>G27/G28</f>
+        <v/>
+      </c>
+      <c r="H29" s="38">
+        <f>H27/H28</f>
+        <v/>
+      </c>
+      <c r="I29" s="38">
+        <f>I27/I28</f>
+        <v/>
+      </c>
+      <c r="J29" s="38">
+        <f>J27/J28</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" s="33" t="inlineStr">
         <is>
           <t>Variação de Preço vs. Regime Atual (R$)</t>
         </is>
       </c>
-      <c r="C25" s="37">
-        <f>C24-'Cálculo Regime Atual'!$C$35</f>
-        <v/>
-      </c>
-      <c r="D25" s="37">
-        <f>D24-'Cálculo Regime Atual'!$C$35</f>
-        <v/>
-      </c>
-      <c r="E25" s="37">
-        <f>E24-'Cálculo Regime Atual'!$C$35</f>
-        <v/>
-      </c>
-      <c r="F25" s="37">
-        <f>F24-'Cálculo Regime Atual'!$C$35</f>
-        <v/>
-      </c>
-      <c r="G25" s="37">
-        <f>G24-'Cálculo Regime Atual'!$C$35</f>
-        <v/>
-      </c>
-      <c r="H25" s="37">
-        <f>H24-'Cálculo Regime Atual'!$C$35</f>
-        <v/>
-      </c>
-      <c r="I25" s="37">
-        <f>I24-'Cálculo Regime Atual'!$C$35</f>
-        <v/>
-      </c>
-      <c r="J25" s="37">
-        <f>J24-'Cálculo Regime Atual'!$C$35</f>
-        <v/>
-      </c>
-    </row>
-    <row r="26">
-      <c r="B26" s="33" t="inlineStr">
+      <c r="C30" s="37">
+        <f>C29-'Cálculo Regime Atual'!$C$35</f>
+        <v/>
+      </c>
+      <c r="D30" s="37">
+        <f>D29-'Cálculo Regime Atual'!$C$35</f>
+        <v/>
+      </c>
+      <c r="E30" s="37">
+        <f>E29-'Cálculo Regime Atual'!$C$35</f>
+        <v/>
+      </c>
+      <c r="F30" s="37">
+        <f>F29-'Cálculo Regime Atual'!$C$35</f>
+        <v/>
+      </c>
+      <c r="G30" s="37">
+        <f>G29-'Cálculo Regime Atual'!$C$35</f>
+        <v/>
+      </c>
+      <c r="H30" s="37">
+        <f>H29-'Cálculo Regime Atual'!$C$35</f>
+        <v/>
+      </c>
+      <c r="I30" s="37">
+        <f>I29-'Cálculo Regime Atual'!$C$35</f>
+        <v/>
+      </c>
+      <c r="J30" s="37">
+        <f>J29-'Cálculo Regime Atual'!$C$35</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" s="33" t="inlineStr">
         <is>
           <t>Variação de Preço vs. Regime Atual (%)</t>
         </is>
       </c>
-      <c r="C26" s="39">
-        <f>C24/'Cálculo Regime Atual'!$C$35-1</f>
-        <v/>
-      </c>
-      <c r="D26" s="39">
-        <f>D24/'Cálculo Regime Atual'!$C$35-1</f>
-        <v/>
-      </c>
-      <c r="E26" s="39">
-        <f>E24/'Cálculo Regime Atual'!$C$35-1</f>
-        <v/>
-      </c>
-      <c r="F26" s="39">
-        <f>F24/'Cálculo Regime Atual'!$C$35-1</f>
-        <v/>
-      </c>
-      <c r="G26" s="39">
-        <f>G24/'Cálculo Regime Atual'!$C$35-1</f>
-        <v/>
-      </c>
-      <c r="H26" s="39">
-        <f>H24/'Cálculo Regime Atual'!$C$35-1</f>
-        <v/>
-      </c>
-      <c r="I26" s="39">
-        <f>I24/'Cálculo Regime Atual'!$C$35-1</f>
-        <v/>
-      </c>
-      <c r="J26" s="39">
-        <f>J24/'Cálculo Regime Atual'!$C$35-1</f>
+      <c r="C31" s="39">
+        <f>C29/'Cálculo Regime Atual'!$C$35-1</f>
+        <v/>
+      </c>
+      <c r="D31" s="39">
+        <f>D29/'Cálculo Regime Atual'!$C$35-1</f>
+        <v/>
+      </c>
+      <c r="E31" s="39">
+        <f>E29/'Cálculo Regime Atual'!$C$35-1</f>
+        <v/>
+      </c>
+      <c r="F31" s="39">
+        <f>F29/'Cálculo Regime Atual'!$C$35-1</f>
+        <v/>
+      </c>
+      <c r="G31" s="39">
+        <f>G29/'Cálculo Regime Atual'!$C$35-1</f>
+        <v/>
+      </c>
+      <c r="H31" s="39">
+        <f>H29/'Cálculo Regime Atual'!$C$35-1</f>
+        <v/>
+      </c>
+      <c r="I31" s="39">
+        <f>I29/'Cálculo Regime Atual'!$C$35-1</f>
+        <v/>
+      </c>
+      <c r="J31" s="39">
+        <f>J29/'Cálculo Regime Atual'!$C$35-1</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="7">
     <mergeCell ref="B7:J7"/>
+    <mergeCell ref="B25:J25"/>
     <mergeCell ref="B20:J20"/>
     <mergeCell ref="C4:E4"/>
     <mergeCell ref="B18:J18"/>
@@ -3045,15 +3232,15 @@
         <v/>
       </c>
       <c r="D8" s="28">
-        <f>'Cálculo Reforma 2027-2033'!C24</f>
+        <f>'Cálculo Reforma 2027-2033'!C29</f>
         <v/>
       </c>
       <c r="E8" s="28">
-        <f>'Cálculo Reforma 2027-2033'!C24-'Cálculo Reforma 2027-2033'!$C$24</f>
+        <f>'Cálculo Reforma 2027-2033'!C29-'Cálculo Reforma 2027-2033'!$C$29</f>
         <v/>
       </c>
       <c r="F8" s="39">
-        <f>'Cálculo Reforma 2027-2033'!C24/'Cálculo Reforma 2027-2033'!$C$24-1</f>
+        <f>'Cálculo Reforma 2027-2033'!C29/'Cálculo Reforma 2027-2033'!$C$29-1</f>
         <v/>
       </c>
     </row>
@@ -3067,15 +3254,15 @@
         <v/>
       </c>
       <c r="D9" s="43">
-        <f>'Cálculo Reforma 2027-2033'!D24</f>
+        <f>'Cálculo Reforma 2027-2033'!D29</f>
         <v/>
       </c>
       <c r="E9" s="43">
-        <f>'Cálculo Reforma 2027-2033'!D24-'Cálculo Reforma 2027-2033'!$C$24</f>
+        <f>'Cálculo Reforma 2027-2033'!D29-'Cálculo Reforma 2027-2033'!$C$29</f>
         <v/>
       </c>
       <c r="F9" s="44">
-        <f>'Cálculo Reforma 2027-2033'!D24/'Cálculo Reforma 2027-2033'!$C$24-1</f>
+        <f>'Cálculo Reforma 2027-2033'!D29/'Cálculo Reforma 2027-2033'!$C$29-1</f>
         <v/>
       </c>
     </row>
@@ -3089,15 +3276,15 @@
         <v/>
       </c>
       <c r="D10" s="28">
-        <f>'Cálculo Reforma 2027-2033'!E24</f>
+        <f>'Cálculo Reforma 2027-2033'!E29</f>
         <v/>
       </c>
       <c r="E10" s="28">
-        <f>'Cálculo Reforma 2027-2033'!E24-'Cálculo Reforma 2027-2033'!$C$24</f>
+        <f>'Cálculo Reforma 2027-2033'!E29-'Cálculo Reforma 2027-2033'!$C$29</f>
         <v/>
       </c>
       <c r="F10" s="39">
-        <f>'Cálculo Reforma 2027-2033'!E24/'Cálculo Reforma 2027-2033'!$C$24-1</f>
+        <f>'Cálculo Reforma 2027-2033'!E29/'Cálculo Reforma 2027-2033'!$C$29-1</f>
         <v/>
       </c>
     </row>
@@ -3111,15 +3298,15 @@
         <v/>
       </c>
       <c r="D11" s="43">
-        <f>'Cálculo Reforma 2027-2033'!F24</f>
+        <f>'Cálculo Reforma 2027-2033'!F29</f>
         <v/>
       </c>
       <c r="E11" s="43">
-        <f>'Cálculo Reforma 2027-2033'!F24-'Cálculo Reforma 2027-2033'!$C$24</f>
+        <f>'Cálculo Reforma 2027-2033'!F29-'Cálculo Reforma 2027-2033'!$C$29</f>
         <v/>
       </c>
       <c r="F11" s="44">
-        <f>'Cálculo Reforma 2027-2033'!F24/'Cálculo Reforma 2027-2033'!$C$24-1</f>
+        <f>'Cálculo Reforma 2027-2033'!F29/'Cálculo Reforma 2027-2033'!$C$29-1</f>
         <v/>
       </c>
     </row>
@@ -3133,15 +3320,15 @@
         <v/>
       </c>
       <c r="D12" s="28">
-        <f>'Cálculo Reforma 2027-2033'!G24</f>
+        <f>'Cálculo Reforma 2027-2033'!G29</f>
         <v/>
       </c>
       <c r="E12" s="28">
-        <f>'Cálculo Reforma 2027-2033'!G24-'Cálculo Reforma 2027-2033'!$C$24</f>
+        <f>'Cálculo Reforma 2027-2033'!G29-'Cálculo Reforma 2027-2033'!$C$29</f>
         <v/>
       </c>
       <c r="F12" s="39">
-        <f>'Cálculo Reforma 2027-2033'!G24/'Cálculo Reforma 2027-2033'!$C$24-1</f>
+        <f>'Cálculo Reforma 2027-2033'!G29/'Cálculo Reforma 2027-2033'!$C$29-1</f>
         <v/>
       </c>
     </row>
@@ -3155,15 +3342,15 @@
         <v/>
       </c>
       <c r="D13" s="43">
-        <f>'Cálculo Reforma 2027-2033'!H24</f>
+        <f>'Cálculo Reforma 2027-2033'!H29</f>
         <v/>
       </c>
       <c r="E13" s="43">
-        <f>'Cálculo Reforma 2027-2033'!H24-'Cálculo Reforma 2027-2033'!$C$24</f>
+        <f>'Cálculo Reforma 2027-2033'!H29-'Cálculo Reforma 2027-2033'!$C$29</f>
         <v/>
       </c>
       <c r="F13" s="44">
-        <f>'Cálculo Reforma 2027-2033'!H24/'Cálculo Reforma 2027-2033'!$C$24-1</f>
+        <f>'Cálculo Reforma 2027-2033'!H29/'Cálculo Reforma 2027-2033'!$C$29-1</f>
         <v/>
       </c>
     </row>
@@ -3177,15 +3364,15 @@
         <v/>
       </c>
       <c r="D14" s="28">
-        <f>'Cálculo Reforma 2027-2033'!I24</f>
+        <f>'Cálculo Reforma 2027-2033'!I29</f>
         <v/>
       </c>
       <c r="E14" s="28">
-        <f>'Cálculo Reforma 2027-2033'!I24-'Cálculo Reforma 2027-2033'!$C$24</f>
+        <f>'Cálculo Reforma 2027-2033'!I29-'Cálculo Reforma 2027-2033'!$C$29</f>
         <v/>
       </c>
       <c r="F14" s="39">
-        <f>'Cálculo Reforma 2027-2033'!I24/'Cálculo Reforma 2027-2033'!$C$24-1</f>
+        <f>'Cálculo Reforma 2027-2033'!I29/'Cálculo Reforma 2027-2033'!$C$29-1</f>
         <v/>
       </c>
     </row>
@@ -3199,15 +3386,15 @@
         <v/>
       </c>
       <c r="D15" s="43">
-        <f>'Cálculo Reforma 2027-2033'!J24</f>
+        <f>'Cálculo Reforma 2027-2033'!J29</f>
         <v/>
       </c>
       <c r="E15" s="43">
-        <f>'Cálculo Reforma 2027-2033'!J24-'Cálculo Reforma 2027-2033'!$C$24</f>
+        <f>'Cálculo Reforma 2027-2033'!J29-'Cálculo Reforma 2027-2033'!$C$29</f>
         <v/>
       </c>
       <c r="F15" s="44">
-        <f>'Cálculo Reforma 2027-2033'!J24/'Cálculo Reforma 2027-2033'!$C$24-1</f>
+        <f>'Cálculo Reforma 2027-2033'!J29/'Cálculo Reforma 2027-2033'!$C$29-1</f>
         <v/>
       </c>
     </row>
@@ -3234,7 +3421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:B38"/>
+  <dimension ref="B2:B39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -3430,36 +3617,43 @@
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="B34" s="45" t="inlineStr">
+    <row r="33" ht="150" customHeight="1">
+      <c r="B33" s="7" t="inlineStr">
+        <is>
+          <t>• Crédito Presumido — Resíduos Sólidos (Art. 170, LC 214/2025): contribuinte do IBS/CBS no regime regular que adquire resíduos sólidos de coletores incentivados (catador pessoa física, cooperativa ou associação de catadores) para destinação final ambientalmente adequada pode apropriar crédito presumido mesmo sem tributação na etapa anterior (o catador normalmente não é contribuinte). Percentuais: CBS fixo em 7% (a partir de 2027); IBS escalonado de 1,3% (2029) a 13% (2033), acompanhando o cronograma geral de transição. Há exclusões no §3º do art. 170 (ex.: agrotóxicos, medicamentos, pilhas e baterias). Modelado na aba 'Cálculo Reforma 2027-2033' apenas quando o campo correspondente em 'Dados de Entrada' for preenchido — aplicável a clientes do setor de reciclagem/sucata; nos demais casos o valor é zero. Este é apenas UM entre vários créditos presumidos setoriais previstos na LC 214/2025 (há também regimes específicos para agronegócio, entre outros); casos não cobertos por esta planilha devem ser analisados individualmente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="B35" s="45" t="inlineStr">
         <is>
           <t>5. RECOMENDAÇÕES AO CONSULTOR</t>
         </is>
       </c>
     </row>
-    <row r="35" ht="30" customHeight="1">
-      <c r="B35" s="7" t="inlineStr">
+    <row r="36" ht="30" customHeight="1">
+      <c r="B36" s="7" t="inlineStr">
         <is>
           <t>• Revisar e atualizar a aba 'Parâmetros' periodicamente, especialmente após publicação das alíquotas de referência pelo Senado Federal e das definições do Comitê Gestor do IBS.</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="45" customHeight="1">
-      <c r="B36" s="7" t="inlineStr">
-        <is>
-          <t>• Para clientes do Simples Nacional com forte relacionamento B2B (vendas para empresas do regime regular), avaliar a conveniência da opção pelo regime de apuração regular do IBS/CBS, dado o potencial de perda de competitividade caso concorrentes ofereçam crédito integral.</t>
         </is>
       </c>
     </row>
     <row r="37" ht="45" customHeight="1">
       <c r="B37" s="7" t="inlineStr">
         <is>
+          <t>• Para clientes do Simples Nacional com forte relacionamento B2B (vendas para empresas do regime regular), avaliar a conveniência da opção pelo regime de apuração regular do IBS/CBS, dado o potencial de perda de competitividade caso concorrentes ofereçam crédito integral.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="45" customHeight="1">
+      <c r="B38" s="7" t="inlineStr">
+        <is>
           <t>• Reavaliar a composição de custos e despesas (aba 'Dados de Entrada') anualmente, pois a Reforma tende a alterar a decisão de compra 'com nota' vs. 'sem nota' (créditos só existem com documentação fiscal idônea).</t>
         </is>
       </c>
     </row>
-    <row r="38" ht="30" customHeight="1">
-      <c r="B38" s="7" t="inlineStr">
+    <row r="39" ht="30" customHeight="1">
+      <c r="B39" s="7" t="inlineStr">
         <is>
           <t>• Esta planilha é uma ferramenta de simulação gerencial: não substitui a apuração fiscal formal, o parecer tributário individualizado nem o acompanhamento da regulamentação infralegal em curso até 2033.</t>
         </is>

</xml_diff>

<commit_message>
Adiciona módulo Simples Nacional: Regime Único x Regime Híbrido (LC 214/2025)
Nova aba "Simples - Único x Híbrido" com ferramenta de decisão para clientes
do Simples Nacional sobre optar pelo regime híbrido de apuração do IBS/CBS
(art. 41, §3º, LC 214/2025): alíquota efetiva atual, componente IBS/CBS já
embutido no DAS, ganho de crédito ao comprador B2B, impacto na carga
tributária do próprio optante, quadro de cenários por mix de carteira,
alertas de restrição (MEI, trava de 2 anos por ressarcimento de bens de
capital) e leitura indicativa. Documentado na Memória de Cálculo.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018ED9zBe28yKRAx5U4xtcTG
</commit_message>
<xml_diff>
--- a/Precificacao_Tributaria_Reforma_2027_2033.xlsx
+++ b/Precificacao_Tributaria_Reforma_2027_2033.xlsx
@@ -13,7 +13,8 @@
     <sheet name="Cálculo Regime Atual" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Cálculo Reforma 2027-2033" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Comparativo Consolidado" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Memória de Cálculo" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Simples - Único x Híbrido" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Memória de Cálculo" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -214,7 +215,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="46">
+  <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -294,6 +295,9 @@
     <xf numFmtId="10" fontId="5" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="5" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="5" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="4" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -940,7 +944,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:F29"/>
+  <dimension ref="B2:F30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -1047,107 +1051,115 @@
     <row r="16" ht="28" customHeight="1">
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>6. Aba 'Memória de Cálculo': documenta fórmulas, premissas, fontes legais e observações técnicas.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="20" customHeight="1">
-      <c r="B18" s="6" t="inlineStr">
+          <t>6. Aba 'Simples - Único x Híbrido': exclusiva para clientes do Simples Nacional — compara o Regime Único (IBS/CBS por dentro do DAS) com o Regime Híbrido (por fora, crédito pleno ao comprador B2B), conforme LC 214/2025, art. 41 §3º.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="28" customHeight="1">
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>7. Aba 'Memória de Cálculo': documenta fórmulas, premissas, fontes legais e observações técnicas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="20" customHeight="1">
+      <c r="B19" s="6" t="inlineStr">
         <is>
           <t>LEGENDA DE CORES</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="B19" s="8" t="inlineStr">
+    <row r="20">
+      <c r="B20" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">  Exemplo  </t>
         </is>
       </c>
-      <c r="C19" s="9" t="inlineStr">
+      <c r="C20" s="9" t="inlineStr">
         <is>
           <t>Célula de entrada — edite aqui</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="B20" s="10" t="inlineStr">
+    <row r="21">
+      <c r="B21" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">  Exemplo  </t>
         </is>
       </c>
-      <c r="C20" s="9" t="inlineStr">
+      <c r="C21" s="9" t="inlineStr">
         <is>
           <t>Fórmula — não editar</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="B21" s="11" t="inlineStr">
+    <row r="22">
+      <c r="B22" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  Exemplo  </t>
         </is>
       </c>
-      <c r="C21" s="9" t="inlineStr">
+      <c r="C22" s="9" t="inlineStr">
         <is>
           <t>Link/referência para outra aba</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="B22" s="12" t="inlineStr">
+    <row r="23">
+      <c r="B23" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">  Exemplo  </t>
         </is>
       </c>
-      <c r="C22" s="9" t="inlineStr">
+      <c r="C23" s="9" t="inlineStr">
         <is>
           <t>Premissa-chave / estimativa a confirmar na regulamentação</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="B23" s="13" t="inlineStr">
+    <row r="24">
+      <c r="B24" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">  Exemplo  </t>
         </is>
       </c>
-      <c r="C23" s="9" t="inlineStr">
+      <c r="C24" s="9" t="inlineStr">
         <is>
           <t>Resultado / total</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="20" customHeight="1">
-      <c r="B25" s="6" t="inlineStr">
+    <row r="26" ht="20" customHeight="1">
+      <c r="B26" s="6" t="inlineStr">
         <is>
           <t>AVISO IMPORTANTE</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="18" customHeight="1">
-      <c r="B26" s="7" t="inlineStr">
+    <row r="27" ht="18" customHeight="1">
+      <c r="B27" s="7" t="inlineStr">
         <is>
           <t>As alíquotas de referência da CBS e do IBS ainda dependem de regulamentação final (Resolução do Senado Federal, nos termos do art. 156-A e art. 195, V, da CF/88, com redação da EC 132/2023, e da LC 214/2025). Os percentuais aqui utilizados são ESTIMATIVAS técnicas (Ministério da Fazenda / IFI, 2024-2025) para fins de simulação e devem ser atualizados pelo contador assim que os valores oficiais forem publicados. Esta planilha é uma ferramenta de apoio gerencial e não substitui a apuração fiscal formal.</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="18" customHeight="1"/>
     <row r="28" ht="18" customHeight="1"/>
     <row r="29" ht="18" customHeight="1"/>
+    <row r="30" ht="18" customHeight="1"/>
   </sheetData>
-  <mergeCells count="12">
+  <mergeCells count="13">
     <mergeCell ref="B4:F4"/>
     <mergeCell ref="B12:F12"/>
-    <mergeCell ref="B26:F29"/>
+    <mergeCell ref="B26:F26"/>
     <mergeCell ref="B16:F16"/>
     <mergeCell ref="B15:F15"/>
     <mergeCell ref="B2:F3"/>
     <mergeCell ref="B11:F11"/>
     <mergeCell ref="B10:F10"/>
-    <mergeCell ref="B25:F25"/>
+    <mergeCell ref="B19:F19"/>
+    <mergeCell ref="B27:F30"/>
     <mergeCell ref="B14:F14"/>
-    <mergeCell ref="B18:F18"/>
+    <mergeCell ref="B17:F17"/>
     <mergeCell ref="B13:F13"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3421,7 +3433,628 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:B39"/>
+  <dimension ref="B2:F57"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <cols>
+    <col width="3" customWidth="1" min="1" max="1"/>
+    <col width="46" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="46" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="2" ht="24" customHeight="1">
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>SIMPLES NACIONAL — REGIME ÚNICO x REGIME HÍBRIDO (LC 214/2025)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="26" customHeight="1">
+      <c r="B3" s="16" t="inlineStr">
+        <is>
+          <t>Aplicável somente se o Regime Tributário em 'Dados de Entrada' for Simples Nacional. Ferramenta de apoio à decisão — não substitui parecer individualizado.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="20" customHeight="1">
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>1. DADOS DO CLIENTE (SIMPLES NACIONAL)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="18" customHeight="1">
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>Anexo do Simples Nacional</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="D6" s="16" t="inlineStr">
+        <is>
+          <t>I=Comércio, II=Indústria, III=Serviços (Fator R), IV=Serviços (CPP à parte), V=Serviços (Fator R&lt;28%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="18" customHeight="1">
+      <c r="B7" s="9" t="inlineStr">
+        <is>
+          <t>RBT12 — Receita Bruta Acumulada 12 Meses (R$)</t>
+        </is>
+      </c>
+      <c r="C7" s="22" t="n">
+        <v>1200000</v>
+      </c>
+    </row>
+    <row r="8" ht="26" customHeight="1">
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>Alíquota Nominal da Faixa (%)</t>
+        </is>
+      </c>
+      <c r="C8" s="21" t="n">
+        <v>0.19</v>
+      </c>
+      <c r="D8" s="16" t="inlineStr">
+        <is>
+          <t>Consultar tabela oficial da faixa/Anexo aplicável (LC 123/2006, Anexos I a V, Portal do Simples Nacional).</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="18" customHeight="1">
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t>Parcela a Deduzir da Faixa (R$)</t>
+        </is>
+      </c>
+      <c r="C9" s="22" t="n">
+        <v>22500</v>
+      </c>
+    </row>
+    <row r="10" ht="34" customHeight="1">
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>% do Anexo correspondente a ICMS/ISS/PIS/COFINS</t>
+        </is>
+      </c>
+      <c r="C10" s="45" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="D10" s="16" t="inlineStr">
+        <is>
+          <t>ESTIMATIVA — usar a tabela de repartição percentual do Anexo/faixa aplicável (LC 123/2006). É a parcela da alíquota efetiva que hoje corresponde aos tributos substituídos por IBS/CBS.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="20" customHeight="1">
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>2. REGIME ÚNICO (HOJE) — ALÍQUOTA EFETIVA E CRÉDITO GERADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Alíquota Efetiva = (RBT12×AlíqNominal − ParcDeduzir) / RBT12</t>
+        </is>
+      </c>
+      <c r="C13" s="18">
+        <f>(C7*C8-C9)/C7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>Carga Tributária Anual — Regime Único (R$)</t>
+        </is>
+      </c>
+      <c r="C14" s="23">
+        <f>C7*C13</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>Componente IBS/CBS Embutido na Alíquota Efetiva (%)</t>
+        </is>
+      </c>
+      <c r="C15" s="27">
+        <f>C13*C10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>Componente IBS/CBS Embutido — valor anual (R$)</t>
+        </is>
+      </c>
+      <c r="C16" s="28">
+        <f>C7*C15</f>
+        <v/>
+      </c>
+      <c r="D16" s="16" t="inlineStr">
+        <is>
+          <t>É o crédito que o cliente PJ comprador já consegue aproveitar HOJE, mesmo no Regime Único.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="20" customHeight="1">
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t>3. PERFIL DA CARTEIRA E ALÍQUOTA DE REFERÊNCIA DA REFORMA</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="26" customHeight="1">
+      <c r="B19" s="9" t="inlineStr">
+        <is>
+          <t>% de Vendas para PJ do Lucro Real/Presumido (B2B com crédito)</t>
+        </is>
+      </c>
+      <c r="C19" s="21" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D19" s="16" t="inlineStr">
+        <is>
+          <t>Vendas para PJ também optante do Simples não geram ganho de crédito no Híbrido — não incluir nesse percentual.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="26" customHeight="1">
+      <c r="B20" s="9" t="inlineStr">
+        <is>
+          <t>Redução Setorial de Alíquota (0% / 30% / 60% / 100%)</t>
+        </is>
+      </c>
+      <c r="C20" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="D20" s="16" t="inlineStr">
+        <is>
+          <t>Preencher se o setor tiver redução prevista na LC 214/2025 (ex.: profissionais de conselho, saúde, educação, cesta básica etc.).</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Alíquota de Referência Cheia (IVA Dual — CBS+IBS)</t>
+        </is>
+      </c>
+      <c r="C21" s="26">
+        <f>Parâmetros!C21</f>
+        <v/>
+      </c>
+      <c r="D21" s="16" t="inlineStr">
+        <is>
+          <t>ESTIMATIVA — não definitiva; depende de Resolução do Senado (LC 214/2025, art. 14).</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>Alíquota de Referência Aplicável (após redução setorial)</t>
+        </is>
+      </c>
+      <c r="C22" s="18">
+        <f>C21*(1-C20)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24" ht="20" customHeight="1">
+      <c r="B24" s="6" t="inlineStr">
+        <is>
+          <t>4. IMPACTO NO COMPRADOR — GANHO DE COMPETITIVIDADE (HÍBRIDO)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" s="9" t="inlineStr">
+        <is>
+          <t>Receita Anual de Vendas B2B (R$)</t>
+        </is>
+      </c>
+      <c r="C25" s="28">
+        <f>C7*C19</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>Crédito Pleno Gerado no Híbrido (R$/ano)</t>
+        </is>
+      </c>
+      <c r="C26" s="28">
+        <f>C25*C22</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" s="9" t="inlineStr">
+        <is>
+          <t>Crédito Hoje sobre a mesma Receita B2B — Regime Único (R$/ano)</t>
+        </is>
+      </c>
+      <c r="C27" s="28">
+        <f>C25*C15</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>GANHO DE CRÉDITO AO COMPRADOR (R$/ano)</t>
+        </is>
+      </c>
+      <c r="C28" s="23">
+        <f>C26-C27</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" s="9" t="inlineStr">
+        <is>
+          <t>Ganho de Crédito sobre a Receita B2B (%)</t>
+        </is>
+      </c>
+      <c r="C29" s="39">
+        <f>IF(C25=0,0,C28/C25)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31" ht="20" customHeight="1">
+      <c r="B31" s="6" t="inlineStr">
+        <is>
+          <t>5. IMPACTO NO PRÓPRIO OPTANTE — CARGA TRIBUTÁRIA DIRETA (HÍBRIDO)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="B32" s="9" t="inlineStr">
+        <is>
+          <t>Compras/Insumos Sujeitos a Crédito no Híbrido (R$/ano)</t>
+        </is>
+      </c>
+      <c r="C32" s="22" t="n">
+        <v>500000</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" s="9" t="inlineStr">
+        <is>
+          <t>% de Aproveitamento do Crédito sobre as Compras</t>
+        </is>
+      </c>
+      <c r="C33" s="21" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="B34" s="9" t="inlineStr">
+        <is>
+          <t>Créditos Tomados nas Compras (R$/ano)</t>
+        </is>
+      </c>
+      <c r="C34" s="28">
+        <f>C32*C33*C22</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="B35" s="9" t="inlineStr">
+        <is>
+          <t>Débito Total de IBS/CBS sobre a Receita Total (R$/ano)</t>
+        </is>
+      </c>
+      <c r="C35" s="28">
+        <f>C7*C22</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="B36" s="9" t="inlineStr">
+        <is>
+          <t>Carga Líquida de IBS/CBS no Híbrido (Débito − Créditos) (R$/ano)</t>
+        </is>
+      </c>
+      <c r="C36" s="28">
+        <f>C35-C34</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="B37" s="9" t="inlineStr">
+        <is>
+          <t>Alíquota Efetiva do DAS sem o Componente IBS/CBS (%)</t>
+        </is>
+      </c>
+      <c r="C37" s="27">
+        <f>C13-C15</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="B38" s="9" t="inlineStr">
+        <is>
+          <t>Demais Tributos do DAS no Híbrido — IRPJ/CSLL/CPP/etc. (R$/ano)</t>
+        </is>
+      </c>
+      <c r="C38" s="28">
+        <f>C7*C37</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t>CARGA TRIBUTÁRIA TOTAL — REGIME HÍBRIDO (R$/ano)</t>
+        </is>
+      </c>
+      <c r="C39" s="23">
+        <f>C38+C36</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>Impacto Líquido para o Optante — Híbrido vs. Único (R$/ano)</t>
+        </is>
+      </c>
+      <c r="C40" s="23">
+        <f>C39-C14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41" ht="30" customHeight="1">
+      <c r="B41" s="9" t="inlineStr">
+        <is>
+          <t>Impacto Líquido para o Optante (%)</t>
+        </is>
+      </c>
+      <c r="C41" s="39">
+        <f>IF(C14=0,0,C40/C14)</f>
+        <v/>
+      </c>
+      <c r="D41" s="16" t="inlineStr">
+        <is>
+          <t>Positivo = carga própria aumenta no Híbrido; negativo = carga própria diminui. Custo de compliance adicional (sistemas, EFD própria, split payment) não está quantificado aqui — avaliar qualitativamente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="20" customHeight="1">
+      <c r="B43" s="6" t="inlineStr">
+        <is>
+          <t>6. QUADRO COMPARATIVO — CENÁRIOS DE MIX DE CARTEIRA</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="30" customHeight="1">
+      <c r="B44" s="14" t="inlineStr">
+        <is>
+          <t>Cenário</t>
+        </is>
+      </c>
+      <c r="C44" s="14" t="inlineStr">
+        <is>
+          <t>% B2B</t>
+        </is>
+      </c>
+      <c r="D44" s="14" t="inlineStr">
+        <is>
+          <t>Ganho de Crédito
+ao Comprador (R$)</t>
+        </is>
+      </c>
+      <c r="E44" s="14" t="inlineStr">
+        <is>
+          <t>Impacto Líquido
+no Optante (R$)</t>
+        </is>
+      </c>
+      <c r="F44" s="14" t="inlineStr">
+        <is>
+          <t>Leitura</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="18" customHeight="1">
+      <c r="B45" s="9" t="inlineStr">
+        <is>
+          <t>B2C Majoritário</t>
+        </is>
+      </c>
+      <c r="C45" s="21" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="D45" s="28">
+        <f>(C7*C45)*C22-(C7*C45)*C15</f>
+        <v/>
+      </c>
+      <c r="E45" s="28">
+        <f>C40</f>
+        <v/>
+      </c>
+      <c r="F45" s="46">
+        <f>IF(D45&gt;0,"Híbrido melhora crédito do comprador","Sem ganho relevante de crédito")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46" ht="18" customHeight="1">
+      <c r="B46" s="9" t="inlineStr">
+        <is>
+          <t>Carteira Mista</t>
+        </is>
+      </c>
+      <c r="C46" s="21" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D46" s="28">
+        <f>(C7*C46)*C22-(C7*C46)*C15</f>
+        <v/>
+      </c>
+      <c r="E46" s="28">
+        <f>C40</f>
+        <v/>
+      </c>
+      <c r="F46" s="46">
+        <f>IF(D46&gt;0,"Híbrido melhora crédito do comprador","Sem ganho relevante de crédito")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47" ht="18" customHeight="1">
+      <c r="B47" s="9" t="inlineStr">
+        <is>
+          <t>B2B Majoritário</t>
+        </is>
+      </c>
+      <c r="C47" s="21" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="D47" s="28">
+        <f>(C7*C47)*C22-(C7*C47)*C15</f>
+        <v/>
+      </c>
+      <c r="E47" s="28">
+        <f>C40</f>
+        <v/>
+      </c>
+      <c r="F47" s="46">
+        <f>IF(D47&gt;0,"Híbrido melhora crédito do comprador","Sem ganho relevante de crédito")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49" ht="26" customHeight="1">
+      <c r="B49" s="16" t="inlineStr">
+        <is>
+          <t>Nota: a coluna 'Impacto Líquido no Optante' usa os mesmos insumos/créditos informados na Seção 5 (não varia por cenário) — refina-se manualmente se as compras também mudarem de composição.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="20" customHeight="1">
+      <c r="B51" s="6" t="inlineStr">
+        <is>
+          <t>7. RESTRIÇÕES E ALERTAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="26" customHeight="1">
+      <c r="B52" s="9" t="inlineStr">
+        <is>
+          <t>Optante é MEI? (Sim/Não)</t>
+        </is>
+      </c>
+      <c r="C52" s="4" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="D52" s="46">
+        <f>IF(C52="Sim","ALERTA: MEI não tem acesso ao Regime Híbrido (Anexo VII, LC 123/2006) — nunca gera crédito pleno a clientes PJ.","")</f>
+        <v/>
+      </c>
+      <c r="E52" s="30" t="n"/>
+      <c r="F52" s="31" t="n"/>
+    </row>
+    <row r="53" ht="30" customHeight="1">
+      <c r="B53" s="7" t="inlineStr">
+        <is>
+          <t>Pretende pedir ressarcimento de crédito sobre bens de capital em 24 meses? (Sim/Não)</t>
+        </is>
+      </c>
+      <c r="C53" s="4" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="D53" s="46">
+        <f>IF(C53="Sim","ALERTA: pedido de ressarcimento de crédito sobre bens de capital trava o retorno ao Regime Único por 2 anos consecutivos.","")</f>
+        <v/>
+      </c>
+      <c r="E53" s="30" t="n"/>
+      <c r="F53" s="31" t="n"/>
+    </row>
+    <row r="54" ht="30" customHeight="1">
+      <c r="B54" s="16" t="inlineStr">
+        <is>
+          <t>Janela de opção: setembro/2026 (vigência 1º sem/2027); março/2027 (vigência 2º sem/2027); a partir daí, opção semestral. Silêncio do contribuinte = permanece no Regime Único. CNPJs abertos entre out/2026 e dez/2026 optam no próprio ato de inscrição.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="20" customHeight="1">
+      <c r="B56" s="6" t="inlineStr">
+        <is>
+          <t>8. LEITURA INDICATIVA (NÃO SUBSTITUI PARECER INDIVIDUALIZADO)</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="24" customHeight="1">
+      <c r="B57" s="47">
+        <f>IF(C52="Sim","MEI: Regime Híbrido não é aplicável.",IF(AND(C19&gt;=0.5,C40&lt;=0),"Carteira majoritariamente B2B e impacto próprio neutro/favorável — avaliar migração para o Híbrido, considerando custo de compliance.",IF(C19&lt;0.3,"Carteira majoritariamente B2C — ganho de crédito tende a ser pouco relevante; Regime Único provavelmente mais vantajoso.","Cenário intermediário — avaliar caso a caso o custo de compliance frente ao ganho de crédito e ao impacto na carga própria.")))</f>
+        <v/>
+      </c>
+      <c r="C57" s="30" t="n"/>
+      <c r="D57" s="30" t="n"/>
+      <c r="E57" s="30" t="n"/>
+      <c r="F57" s="31" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="23">
+    <mergeCell ref="B54:F54"/>
+    <mergeCell ref="D41:F41"/>
+    <mergeCell ref="B3:F3"/>
+    <mergeCell ref="B31:F31"/>
+    <mergeCell ref="D53:F53"/>
+    <mergeCell ref="B18:F18"/>
+    <mergeCell ref="D16:F16"/>
+    <mergeCell ref="B56:F56"/>
+    <mergeCell ref="B43:F43"/>
+    <mergeCell ref="B12:F12"/>
+    <mergeCell ref="B2:F2"/>
+    <mergeCell ref="D8:F8"/>
+    <mergeCell ref="B57:F57"/>
+    <mergeCell ref="D20:F20"/>
+    <mergeCell ref="B49:F49"/>
+    <mergeCell ref="D10:F10"/>
+    <mergeCell ref="D19:F19"/>
+    <mergeCell ref="B24:F24"/>
+    <mergeCell ref="B5:F5"/>
+    <mergeCell ref="B51:F51"/>
+    <mergeCell ref="D52:F52"/>
+    <mergeCell ref="D21:F21"/>
+    <mergeCell ref="D6:F6"/>
+  </mergeCells>
+  <dataValidations count="2">
+    <dataValidation sqref="C6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"I,II,III,IV,V"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C52 C53" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"Sim,Não"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B2:B50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -3436,7 +4069,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="B4" s="45" t="inlineStr">
+      <c r="B4" s="48" t="inlineStr">
         <is>
           <t>1. BASE LEGAL</t>
         </is>
@@ -3463,199 +4096,269 @@
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="B9" s="45" t="inlineStr">
+    <row r="8" ht="45" customHeight="1">
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>• LC 214/2025, art. 41, §3º — permite ao optante do Simples Nacional escolher, semestralmente, entre recolher IBS/CBS dentro do DAS (Regime Único) ou por fora, pelas regras gerais do regime não cumulativo (Regime Híbrido). Resolução CGSN nº 183/2025 operacionaliza a opção no âmbito do Simples.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="48" t="inlineStr">
         <is>
           <t>2. METODOLOGIA APLICADA</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="15" customHeight="1">
-      <c r="B10" s="7" t="inlineStr">
-        <is>
-          <t>1) Identificação da atividade e do tipo de operação (mercadoria/serviço) — aba 'Dados de Entrada'.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="15" customHeight="1">
       <c r="B11" s="7" t="inlineStr">
         <is>
+          <t>1) Identificação da atividade e do tipo de operação (mercadoria/serviço) — aba 'Dados de Entrada'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="15" customHeight="1">
+      <c r="B12" s="7" t="inlineStr">
+        <is>
           <t>2) Identificação do regime tributário do cliente (Simples Nacional, Lucro Presumido ou Lucro Real).</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="30" customHeight="1">
-      <c r="B12" s="7" t="inlineStr">
-        <is>
-          <t>3) Identificação da tributação aplicável em cada esfera (federal: PIS/COFINS/IPI; estadual/municipal: ICMS/ISS) — aba 'Parâmetros'.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="30" customHeight="1">
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>4) Cálculo dos tributos nominais e da carga tributária efetiva do regime atual — aba 'Cálculo Regime Atual'.</t>
+          <t>3) Identificação da tributação aplicável em cada esfera (federal: PIS/COFINS/IPI; estadual/municipal: ICMS/ISS) — aba 'Parâmetros'.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="30" customHeight="1">
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>5) Cálculo dos créditos recuperáveis sobre insumos (não cumulatividade) — reduzem o CUSTO na formação de preço, não a alíquota de débito.</t>
+          <t>4) Cálculo dos tributos nominais e da carga tributária efetiva do regime atual — aba 'Cálculo Regime Atual'.</t>
         </is>
       </c>
     </row>
     <row r="15" ht="30" customHeight="1">
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>6) Aplicação do cronograma de transição da Reforma (pesos ano a ano definidos na EC 132/2023 e LC 214/2025) para obter a carga tributária efetiva de 2026 a 2033 — aba 'Cálculo Reforma 2027-2033'.</t>
+          <t>5) Cálculo dos créditos recuperáveis sobre insumos (não cumulatividade) — reduzem o CUSTO na formação de preço, não a alíquota de débito.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="30" customHeight="1">
       <c r="B16" s="7" t="inlineStr">
         <is>
+          <t>6) Aplicação do cronograma de transição da Reforma (pesos ano a ano definidos na EC 132/2023 e LC 214/2025) para obter a carga tributária efetiva de 2026 a 2033 — aba 'Cálculo Reforma 2027-2033'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="30" customHeight="1">
+      <c r="B17" s="7" t="inlineStr">
+        <is>
           <t>7) Formação do preço de venda pelo método do divisor ('por dentro'): Preço = (Custo − Créditos) ÷ [1 − (%Despesas Variáveis + %Despesas Fixas + %Margem + %Carga Tributária)].</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="15" customHeight="1">
-      <c r="B17" s="7" t="inlineStr">
+    <row r="18" ht="15" customHeight="1">
+      <c r="B18" s="7" t="inlineStr">
         <is>
           <t>8) Comparação dos cenários ano a ano e conclusão — aba 'Comparativo Consolidado'.</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="B19" s="45" t="inlineStr">
+    <row r="20">
+      <c r="B20" s="48" t="inlineStr">
         <is>
           <t>3. FÓRMULA DE FORMAÇÃO DE PREÇO (MÉTODO DO DIVISOR)</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="15" customHeight="1">
-      <c r="B20" s="7" t="inlineStr">
+    <row r="21" ht="15" customHeight="1">
+      <c r="B21" s="7" t="inlineStr">
         <is>
           <t>Preço de Venda = (Custo Total − Créditos Tributários Recuperáveis) ÷ Divisor</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="30" customHeight="1">
-      <c r="B21" s="7" t="inlineStr">
+    <row r="22" ht="30" customHeight="1">
+      <c r="B22" s="7" t="inlineStr">
         <is>
           <t>Divisor = 1 − (% Despesas Variáveis + % Despesas Fixas + % Margem de Lucro Desejada + % Carga Tributária Efetiva)</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="45" customHeight="1">
-      <c r="B22" s="7" t="inlineStr">
+    <row r="23" ht="45" customHeight="1">
+      <c r="B23" s="7" t="inlineStr">
         <is>
           <t>Este método ('markup divisor' ou preço 'por dentro') é o padrão utilizado em custos e formação de preço no Brasil, pois todos os tributos e percentuais informados incidem sobre o próprio preço de venda (base 'por dentro'), e não sobre o custo.</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="B24" s="45" t="inlineStr">
+    <row r="25">
+      <c r="B25" s="48" t="inlineStr">
         <is>
           <t>4. PREMISSAS E SIMPLIFICAÇÕES ADOTADAS</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="60" customHeight="1">
-      <c r="B25" s="7" t="inlineStr">
+    <row r="26" ht="60" customHeight="1">
+      <c r="B26" s="7" t="inlineStr">
         <is>
           <t>• As alíquotas de CBS e IBS constantes da aba 'Parâmetros' são ESTIMATIVAS técnicas (associadas a estudos do Ministério da Fazenda e da Instituição Fiscal Independente — IFI, 2024/2025), pois a alíquota de referência definitiva depende de Resolução do Senado Federal, a ser recalibrada anualmente pelo Comitê Gestor do IBS conforme a arrecadação observada. ATUALIZAR sempre que houver nova publicação oficial.</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="90" customHeight="1">
-      <c r="B26" s="7" t="inlineStr">
+    <row r="27" ht="90" customHeight="1">
+      <c r="B27" s="7" t="inlineStr">
         <is>
           <t>• Simples Nacional: a Reforma preserva o regime unificado do DAS para o optante padrão — a carga tributária própria do optante é modelada como CONSTANTE (alíquota efetiva do Simples) em todo o período 2026-2033, pois PIS/COFINS/ICMS/ISS continuam recolhidos dentro da guia única, sem discriminação de CBS/IBS na apuração do próprio contribuinte. A LC 214/2025 faculta ao optante do Simples migrar para o 'regime de apuração regular' do IBS/CBS caso deseje conceder crédito integral a clientes sujeitos ao regime regular (decisão estratégica a avaliar caso a caso — não modelada automaticamente nesta planilha).</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="60" customHeight="1">
-      <c r="B27" s="7" t="inlineStr">
+    <row r="28" ht="60" customHeight="1">
+      <c r="B28" s="7" t="inlineStr">
         <is>
           <t>• Lucro Presumido: no regime ATUAL, PIS/COFINS são cumulativos (sem crédito). Sob a Reforma, CBS e IBS são não cumulativos de forma ampla, inclusive para o Lucro Presumido — por isso a planilha passa a considerar créditos sobre insumos para esse regime a partir da transição, o que representa um ganho relevante a destacar na análise ao cliente.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="45" customHeight="1">
-      <c r="B28" s="7" t="inlineStr">
-        <is>
-          <t>• IPI: por simplificação, foi tratado dentro do mesmo cronograma de extinção do PIS/COFINS (ambos tributos federais eliminados a partir de 2027, exceto industrialização na Zona Franca de Manaus, que mantém tratamento diferenciado e não está contemplada nesta planilha).</t>
         </is>
       </c>
     </row>
     <row r="29" ht="45" customHeight="1">
       <c r="B29" s="7" t="inlineStr">
         <is>
-          <t>• Imposto Seletivo (IS): modelado apenas quando o produto for sinalizado como sujeito ao IS em 'Dados de Entrada' (ex.: cigarros, bebidas alcoólicas, veículos poluentes, bens minerais). Alíquota específica deve ser pesquisada por NCM/produto e ajustada em 'Parâmetros'.</t>
+          <t>• IPI: por simplificação, foi tratado dentro do mesmo cronograma de extinção do PIS/COFINS (ambos tributos federais eliminados a partir de 2027, exceto industrialização na Zona Franca de Manaus, que mantém tratamento diferenciado e não está contemplada nesta planilha).</t>
         </is>
       </c>
     </row>
     <row r="30" ht="45" customHeight="1">
       <c r="B30" s="7" t="inlineStr">
         <is>
+          <t>• Imposto Seletivo (IS): modelado apenas quando o produto for sinalizado como sujeito ao IS em 'Dados de Entrada' (ex.: cigarros, bebidas alcoólicas, veículos poluentes, bens minerais). Alíquota específica deve ser pesquisada por NCM/produto e ajustada em 'Parâmetros'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="45" customHeight="1">
+      <c r="B31" s="7" t="inlineStr">
+        <is>
           <t>• Créditos tributários: calculados como % de aproveitamento aplicado sobre os insumos elegíveis, multiplicado pela alíquota nominal (regime atual) ou pela carga efetiva do ano (Reforma). Créditos reduzem o CUSTO líquido usado na fórmula do preço — não reduzem a alíquota de débito que compõe o divisor.</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="60" customHeight="1">
-      <c r="B31" s="7" t="inlineStr">
+    <row r="32" ht="60" customHeight="1">
+      <c r="B32" s="7" t="inlineStr">
         <is>
           <t>• Split payment: a LC 214/2025 prevê mecanismo de recolhimento automático do IBS/CBS no momento da liquidação financeira da venda ('split payment'). Esse mecanismo não altera a carga tributária, mas impacta o fluxo de caixa (o valor do tributo é segregado antes de ingressar na conta do vendedor) — recomenda-se atenção ao capital de giro na transição, não quantificada nesta planilha.</t>
         </is>
       </c>
     </row>
-    <row r="32" ht="30" customHeight="1">
-      <c r="B32" s="7" t="inlineStr">
+    <row r="33" ht="30" customHeight="1">
+      <c r="B33" s="7" t="inlineStr">
         <is>
           <t>• Cashback / devolução para famílias de baixa renda e cesta básica nacional (alíquota zero) não foram modelados, pois dependem do enquadramento específico do produto/serviço e do perfil do consumidor final.</t>
         </is>
       </c>
     </row>
-    <row r="33" ht="150" customHeight="1">
-      <c r="B33" s="7" t="inlineStr">
+    <row r="34" ht="150" customHeight="1">
+      <c r="B34" s="7" t="inlineStr">
         <is>
           <t>• Crédito Presumido — Resíduos Sólidos (Art. 170, LC 214/2025): contribuinte do IBS/CBS no regime regular que adquire resíduos sólidos de coletores incentivados (catador pessoa física, cooperativa ou associação de catadores) para destinação final ambientalmente adequada pode apropriar crédito presumido mesmo sem tributação na etapa anterior (o catador normalmente não é contribuinte). Percentuais: CBS fixo em 7% (a partir de 2027); IBS escalonado de 1,3% (2029) a 13% (2033), acompanhando o cronograma geral de transição. Há exclusões no §3º do art. 170 (ex.: agrotóxicos, medicamentos, pilhas e baterias). Modelado na aba 'Cálculo Reforma 2027-2033' apenas quando o campo correspondente em 'Dados de Entrada' for preenchido — aplicável a clientes do setor de reciclagem/sucata; nos demais casos o valor é zero. Este é apenas UM entre vários créditos presumidos setoriais previstos na LC 214/2025 (há também regimes específicos para agronegócio, entre outros); casos não cobertos por esta planilha devem ser analisados individualmente.</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="B35" s="45" t="inlineStr">
+    <row r="36">
+      <c r="B36" s="48" t="inlineStr">
         <is>
           <t>5. RECOMENDAÇÕES AO CONSULTOR</t>
         </is>
       </c>
     </row>
-    <row r="36" ht="30" customHeight="1">
-      <c r="B36" s="7" t="inlineStr">
+    <row r="37" ht="30" customHeight="1">
+      <c r="B37" s="7" t="inlineStr">
         <is>
           <t>• Revisar e atualizar a aba 'Parâmetros' periodicamente, especialmente após publicação das alíquotas de referência pelo Senado Federal e das definições do Comitê Gestor do IBS.</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" ht="45" customHeight="1">
-      <c r="B37" s="7" t="inlineStr">
-        <is>
-          <t>• Para clientes do Simples Nacional com forte relacionamento B2B (vendas para empresas do regime regular), avaliar a conveniência da opção pelo regime de apuração regular do IBS/CBS, dado o potencial de perda de competitividade caso concorrentes ofereçam crédito integral.</t>
         </is>
       </c>
     </row>
     <row r="38" ht="45" customHeight="1">
       <c r="B38" s="7" t="inlineStr">
         <is>
+          <t>• Para clientes do Simples Nacional com forte relacionamento B2B (vendas para empresas do regime regular), avaliar a conveniência da opção pelo regime de apuração regular do IBS/CBS, dado o potencial de perda de competitividade caso concorrentes ofereçam crédito integral.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="45" customHeight="1">
+      <c r="B39" s="7" t="inlineStr">
+        <is>
           <t>• Reavaliar a composição de custos e despesas (aba 'Dados de Entrada') anualmente, pois a Reforma tende a alterar a decisão de compra 'com nota' vs. 'sem nota' (créditos só existem com documentação fiscal idônea).</t>
         </is>
       </c>
     </row>
-    <row r="39" ht="30" customHeight="1">
-      <c r="B39" s="7" t="inlineStr">
+    <row r="40" ht="30" customHeight="1">
+      <c r="B40" s="7" t="inlineStr">
         <is>
           <t>• Esta planilha é uma ferramenta de simulação gerencial: não substitui a apuração fiscal formal, o parecer tributário individualizado nem o acompanhamento da regulamentação infralegal em curso até 2033.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="B42" s="48" t="inlineStr">
+        <is>
+          <t>6. MÓDULO 'SIMPLES — ÚNICO x HÍBRIDO' (LC 214/2025, ART. 41, §3º)</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="45" customHeight="1">
+      <c r="B43" s="7" t="inlineStr">
+        <is>
+          <t>• Objetivo: apoiar a decisão de cliente do Simples Nacional entre permanecer no Regime Único (IBS/CBS recolhidos por dentro do DAS) ou migrar para o Regime Híbrido (IBS/CBS apurados por fora, pelo regime não cumulativo, com repasse de crédito pleno ao comprador).</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="30" customHeight="1">
+      <c r="B44" s="7" t="inlineStr">
+        <is>
+          <t>• Alíquota Efetiva do Simples = (RBT12 × Alíquota Nominal da Faixa − Parcela a Deduzir) ÷ RBT12 (LC 123/2006, art. 18, §1º-A).</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="45" customHeight="1">
+      <c r="B45" s="7" t="inlineStr">
+        <is>
+          <t>• Componente IBS/CBS embutido = Alíquota Efetiva × % do Anexo correspondente a ICMS/ISS/PIS/COFINS. Esse percentual é uma ESTIMATIVA a conferir na tabela de repartição do Anexo/faixa aplicável — não foi cravado como valor fixo na planilha por variar por Anexo e faixa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="30" customHeight="1">
+      <c r="B46" s="7" t="inlineStr">
+        <is>
+          <t>• Crédito pleno no Híbrido = Receita B2B × Alíquota de Referência aplicável (cheia ou reduzida por regime específico do setor). Ganho de crédito ao comprador = Crédito Híbrido − Componente já embutido hoje.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="60" customHeight="1">
+      <c r="B47" s="7" t="inlineStr">
+        <is>
+          <t>• Impacto no próprio optante = compara a carga total no Regime Único com a carga total no Híbrido (demais tributos do DAS sem o componente IBS/CBS + débito de IBS/CBS líquido de créditos sobre compras) — segue o item 5.5 da metodologia de referência, evitando superestimar o custo do Híbrido ao ignorar os créditos que a própria empresa pode tomar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="45" customHeight="1">
+      <c r="B48" s="7" t="inlineStr">
+        <is>
+          <t>• Restrições sempre a observar: MEI não acessa o Regime Híbrido; pedido de ressarcimento de crédito sobre bens de capital trava o retorno ao Regime Único por 2 anos consecutivos; se o comprador PJ também for optante do Simples (Regime Único), o ganho de crédito é irrelevante para ele.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="30" customHeight="1">
+      <c r="B49" s="7" t="inlineStr">
+        <is>
+          <t>• Custo de compliance adicional (sistemas, EFD própria de IBS/CBS, split payment) é apenas qualitativo nesta planilha — não há campo quantitativo, pois depende do porte da estrutura fiscal/ERP de cada cliente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="45" customHeight="1">
+      <c r="B50" s="7" t="inlineStr">
+        <is>
+          <t>• A leitura indicativa da Seção 8 da aba é apenas um sinalizador inicial baseado no % de vendas B2B e no impacto líquido calculado — a decisão final deve considerar também o custo de compliance, o apetite do cliente para complexidade adicional e a janela de opção vigente.</t>
         </is>
       </c>
     </row>

</xml_diff>